<commit_message>
Extender analisis a 9 meses (Ene-Sep) para Calzapato y Kelder
Se agregan Julio, Agosto y Septiembre. La tendencia ahora compara
siempre el trimestre mas reciente contra el inmediato anterior en
vez de la primera mitad contra el resto, para que no se desbalancee
al crecer el numero de meses cargados. Se corrige tambien un bug de
formato de Excel con columnas que contienen NaN (sucursales sin
datos en todos los meses).
</commit_message>
<xml_diff>
--- a/data/raw/Junio.xlsx
+++ b/data/raw/Junio.xlsx
@@ -584,7 +584,7 @@
         <v>0</v>
       </c>
       <c r="R7" s="66">
-        <v>7.69</v>
+        <v>7.14</v>
       </c>
       <c r="S7" s="65">
         <v>100</v>
@@ -1088,7 +1088,7 @@
         <v>0</v>
       </c>
       <c r="R16" s="66">
-        <v>25.00</v>
+        <v>27.27</v>
       </c>
       <c r="S16" s="65">
         <v>0</v>
@@ -1424,7 +1424,7 @@
         <v>0</v>
       </c>
       <c r="R22" s="66">
-        <v>20.00</v>
+        <v>22.22</v>
       </c>
       <c r="S22" s="65">
         <v>0</v>
@@ -1724,20 +1724,20 @@
       </c>
       <c t="inlineStr" r="C28">
         <is>
-          <t xml:space="preserve">073 - GUASAVE CORREGIDORA</t>
+          <t xml:space="preserve">074 - CAMPEON MOCHIS</t>
         </is>
       </c>
       <c r="D28" s="57">
-        <v>0.00</v>
+        <v>2202633.53</v>
       </c>
       <c r="E28" s="57">
-        <v>726194.87</v>
+        <v>2279589.00</v>
       </c>
       <c t="n" r="F28">
-        <v>0.0</v>
-      </c>
-      <c r="H28" s="65">
-        <v>0</v>
+        <v>96.6</v>
+      </c>
+      <c r="H28" s="66">
+        <v>2.01</v>
       </c>
       <c t="inlineStr" r="I28">
         <is>
@@ -1754,19 +1754,19 @@
         <v>100</v>
       </c>
       <c r="O28" s="66">
-        <v>0.00</v>
+        <v>14.22</v>
       </c>
       <c r="P28" s="65">
         <v>0</v>
       </c>
-      <c r="R28" s="65">
-        <v>0</v>
+      <c r="R28" s="66">
+        <v>0.00</v>
       </c>
       <c r="S28" s="65">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="U28" s="65">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="29">
@@ -1780,20 +1780,20 @@
       </c>
       <c t="inlineStr" r="C29">
         <is>
-          <t xml:space="preserve">074 - CAMPEON MOCHIS</t>
+          <t xml:space="preserve">083 - OBREGON PRECIADO</t>
         </is>
       </c>
       <c r="D29" s="57">
-        <v>2202633.53</v>
+        <v>1517325.13</v>
       </c>
       <c r="E29" s="57">
-        <v>2279589.00</v>
+        <v>1750065.00</v>
       </c>
       <c t="n" r="F29">
-        <v>96.6</v>
+        <v>86.7</v>
       </c>
       <c r="H29" s="66">
-        <v>2.01</v>
+        <v>2.27</v>
       </c>
       <c t="inlineStr" r="I29">
         <is>
@@ -1804,16 +1804,16 @@
         <v>0</v>
       </c>
       <c r="L29" s="57">
-        <v>0.00</v>
+        <v>-35828.43</v>
       </c>
       <c r="M29" s="65">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="O29" s="66">
-        <v>14.22</v>
+        <v>22.37</v>
       </c>
       <c r="P29" s="65">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="R29" s="66">
         <v>0.00</v>
@@ -1822,7 +1822,7 @@
         <v>100</v>
       </c>
       <c r="U29" s="65">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="30">
@@ -1836,20 +1836,20 @@
       </c>
       <c t="inlineStr" r="C30">
         <is>
-          <t xml:space="preserve">083 - OBREGON PRECIADO</t>
+          <t xml:space="preserve">088 - Plaza Centenario Mochis</t>
         </is>
       </c>
       <c r="D30" s="57">
-        <v>1517325.13</v>
+        <v>461118.15</v>
       </c>
       <c r="E30" s="57">
-        <v>1750065.00</v>
+        <v>543675.00</v>
       </c>
       <c t="n" r="F30">
-        <v>86.7</v>
+        <v>84.8</v>
       </c>
       <c r="H30" s="66">
-        <v>2.27</v>
+        <v>1.73</v>
       </c>
       <c t="inlineStr" r="I30">
         <is>
@@ -1860,22 +1860,22 @@
         <v>0</v>
       </c>
       <c r="L30" s="57">
-        <v>-35828.43</v>
+        <v>-1969.10</v>
       </c>
       <c r="M30" s="65">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="O30" s="66">
-        <v>22.37</v>
+        <v>-0.08</v>
       </c>
       <c r="P30" s="65">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="R30" s="66">
-        <v>0.00</v>
+        <v>16.67</v>
       </c>
       <c r="S30" s="65">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="U30" s="65">
         <v>2</v>
@@ -1892,20 +1892,20 @@
       </c>
       <c t="inlineStr" r="C31">
         <is>
-          <t xml:space="preserve">088 - Plaza Centenario Mochis</t>
+          <t xml:space="preserve">089 - OBREGON SONORA MERCADO</t>
         </is>
       </c>
       <c r="D31" s="57">
-        <v>461118.15</v>
+        <v>0.00</v>
       </c>
       <c r="E31" s="57">
-        <v>543675.00</v>
-      </c>
-      <c t="n" r="F31">
-        <v>84.8</v>
-      </c>
-      <c r="H31" s="66">
-        <v>1.73</v>
+        <v>0.00</v>
+      </c>
+      <c r="F31" s="65">
+        <v>0</v>
+      </c>
+      <c r="H31" s="65">
+        <v>0</v>
       </c>
       <c t="inlineStr" r="I31">
         <is>
@@ -1916,19 +1916,19 @@
         <v>0</v>
       </c>
       <c r="L31" s="57">
-        <v>-1969.10</v>
+        <v>0.00</v>
       </c>
       <c r="M31" s="65">
         <v>100</v>
       </c>
-      <c r="O31" s="66">
-        <v>-0.08</v>
+      <c r="O31" s="65">
+        <v>0</v>
       </c>
       <c r="P31" s="65">
         <v>0</v>
       </c>
-      <c r="R31" s="66">
-        <v>16.67</v>
+      <c r="R31" s="65">
+        <v>0</v>
       </c>
       <c r="S31" s="65">
         <v>0</v>
@@ -1948,20 +1948,20 @@
       </c>
       <c t="inlineStr" r="C32">
         <is>
-          <t xml:space="preserve">089 - OBREGON SONORA MERCADO</t>
+          <t xml:space="preserve">091 - Guasave Campeon</t>
         </is>
       </c>
       <c r="D32" s="57">
-        <v>0.00</v>
+        <v>758891.03</v>
       </c>
       <c r="E32" s="57">
-        <v>0.00</v>
-      </c>
-      <c r="F32" s="65">
-        <v>0</v>
-      </c>
-      <c r="H32" s="65">
-        <v>0</v>
+        <v>785727.00</v>
+      </c>
+      <c t="n" r="F32">
+        <v>96.6</v>
+      </c>
+      <c r="H32" s="66">
+        <v>1.67</v>
       </c>
       <c t="inlineStr" r="I32">
         <is>
@@ -1972,25 +1972,25 @@
         <v>0</v>
       </c>
       <c r="L32" s="57">
-        <v>0.00</v>
+        <v>-4156.38</v>
       </c>
       <c r="M32" s="65">
-        <v>100</v>
-      </c>
-      <c r="O32" s="65">
-        <v>0</v>
+        <v>0</v>
+      </c>
+      <c r="O32" s="66">
+        <v>11.30</v>
       </c>
       <c r="P32" s="65">
         <v>0</v>
       </c>
-      <c r="R32" s="65">
-        <v>0</v>
+      <c r="R32" s="66">
+        <v>42.86</v>
       </c>
       <c r="S32" s="65">
         <v>0</v>
       </c>
       <c r="U32" s="65">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="33">
@@ -2004,20 +2004,20 @@
       </c>
       <c t="inlineStr" r="C33">
         <is>
-          <t xml:space="preserve">091 - Guasave Campeon</t>
+          <t xml:space="preserve">093 - SAN RAFAEL CLN</t>
         </is>
       </c>
       <c r="D33" s="57">
-        <v>758891.03</v>
+        <v>0.00</v>
       </c>
       <c r="E33" s="57">
-        <v>785727.00</v>
+        <v>842872.95</v>
       </c>
       <c t="n" r="F33">
-        <v>96.6</v>
-      </c>
-      <c r="H33" s="66">
-        <v>1.67</v>
+        <v>0.0</v>
+      </c>
+      <c r="H33" s="65">
+        <v>0</v>
       </c>
       <c t="inlineStr" r="I33">
         <is>
@@ -2028,25 +2028,25 @@
         <v>0</v>
       </c>
       <c r="L33" s="57">
-        <v>-4156.38</v>
+        <v>0.00</v>
       </c>
       <c r="M33" s="65">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="O33" s="66">
-        <v>11.30</v>
+        <v>0.00</v>
       </c>
       <c r="P33" s="65">
         <v>0</v>
       </c>
-      <c r="R33" s="66">
-        <v>42.86</v>
+      <c r="R33" s="65">
+        <v>0</v>
       </c>
       <c r="S33" s="65">
         <v>0</v>
       </c>
       <c r="U33" s="65">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="34">
@@ -2060,20 +2060,20 @@
       </c>
       <c t="inlineStr" r="C34">
         <is>
-          <t xml:space="preserve">093 - SAN RAFAEL CLN</t>
+          <t xml:space="preserve">105 - LA PAZ 16 DE SEPTIEMBRE</t>
         </is>
       </c>
       <c r="D34" s="57">
-        <v>0.00</v>
+        <v>1148289.62</v>
       </c>
       <c r="E34" s="57">
-        <v>842872.95</v>
+        <v>1490458.00</v>
       </c>
       <c t="n" r="F34">
-        <v>0.0</v>
-      </c>
-      <c r="H34" s="65">
-        <v>0</v>
+        <v>77.0</v>
+      </c>
+      <c r="H34" s="66">
+        <v>1.77</v>
       </c>
       <c t="inlineStr" r="I34">
         <is>
@@ -2090,19 +2090,19 @@
         <v>100</v>
       </c>
       <c r="O34" s="66">
-        <v>0.00</v>
+        <v>8.64</v>
       </c>
       <c r="P34" s="65">
         <v>0</v>
       </c>
-      <c r="R34" s="65">
-        <v>0</v>
+      <c r="R34" s="66">
+        <v>0.00</v>
       </c>
       <c r="S34" s="65">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="U34" s="65">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="35">
@@ -2116,20 +2116,20 @@
       </c>
       <c t="inlineStr" r="C35">
         <is>
-          <t xml:space="preserve">105 - LA PAZ 16 DE SEPTIEMBRE</t>
+          <t xml:space="preserve">107 - CONCHITA CLN</t>
         </is>
       </c>
       <c r="D35" s="57">
-        <v>1148289.62</v>
+        <v>620741.50</v>
       </c>
       <c r="E35" s="57">
-        <v>1490458.00</v>
+        <v>1002005.00</v>
       </c>
       <c t="n" r="F35">
-        <v>77.0</v>
-      </c>
-      <c r="H35" s="66">
-        <v>1.77</v>
+        <v>61.9</v>
+      </c>
+      <c t="n" r="H35">
+        <v>1.6</v>
       </c>
       <c t="inlineStr" r="I35">
         <is>
@@ -2146,19 +2146,19 @@
         <v>100</v>
       </c>
       <c r="O35" s="66">
-        <v>8.64</v>
+        <v>1.56</v>
       </c>
       <c r="P35" s="65">
         <v>0</v>
       </c>
       <c r="R35" s="66">
-        <v>0.00</v>
+        <v>14.29</v>
       </c>
       <c r="S35" s="65">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="U35" s="65">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="36">
@@ -2172,20 +2172,20 @@
       </c>
       <c t="inlineStr" r="C36">
         <is>
-          <t xml:space="preserve">107 - CONCHITA CLN</t>
+          <t xml:space="preserve">108 - HERMOSILLO QUIROGA</t>
         </is>
       </c>
       <c r="D36" s="57">
-        <v>620741.50</v>
+        <v>1066827.98</v>
       </c>
       <c r="E36" s="57">
-        <v>1002005.00</v>
+        <v>1438277.00</v>
       </c>
       <c t="n" r="F36">
-        <v>61.9</v>
-      </c>
-      <c t="n" r="H36">
-        <v>1.6</v>
+        <v>74.2</v>
+      </c>
+      <c r="H36" s="66">
+        <v>1.91</v>
       </c>
       <c t="inlineStr" r="I36">
         <is>
@@ -2196,25 +2196,25 @@
         <v>0</v>
       </c>
       <c r="L36" s="57">
-        <v>0.00</v>
+        <v>-2558.84</v>
       </c>
       <c r="M36" s="65">
         <v>100</v>
       </c>
       <c r="O36" s="66">
-        <v>1.56</v>
+        <v>12.12</v>
       </c>
       <c r="P36" s="65">
         <v>0</v>
       </c>
       <c r="R36" s="66">
-        <v>14.29</v>
+        <v>0.00</v>
       </c>
       <c r="S36" s="65">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="U36" s="65">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="37">
@@ -2228,20 +2228,20 @@
       </c>
       <c t="inlineStr" r="C37">
         <is>
-          <t xml:space="preserve">108 - HERMOSILLO QUIROGA</t>
+          <t xml:space="preserve">111 - NAVOLATO ALMADA</t>
         </is>
       </c>
       <c r="D37" s="57">
-        <v>1066827.98</v>
+        <v>641687.56</v>
       </c>
       <c r="E37" s="57">
-        <v>1438277.00</v>
+        <v>996993.00</v>
       </c>
       <c t="n" r="F37">
-        <v>74.2</v>
+        <v>64.4</v>
       </c>
       <c r="H37" s="66">
-        <v>1.91</v>
+        <v>2.05</v>
       </c>
       <c t="inlineStr" r="I37">
         <is>
@@ -2252,13 +2252,13 @@
         <v>0</v>
       </c>
       <c r="L37" s="57">
-        <v>-2558.84</v>
+        <v>0.00</v>
       </c>
       <c r="M37" s="65">
         <v>100</v>
       </c>
       <c r="O37" s="66">
-        <v>12.12</v>
+        <v>-16.95</v>
       </c>
       <c r="P37" s="65">
         <v>0</v>
@@ -2284,20 +2284,20 @@
       </c>
       <c t="inlineStr" r="C38">
         <is>
-          <t xml:space="preserve">111 - NAVOLATO ALMADA</t>
+          <t xml:space="preserve">112 - SORIANA SAN JOSE</t>
         </is>
       </c>
       <c r="D38" s="57">
-        <v>641687.56</v>
+        <v>4022300.51</v>
       </c>
       <c r="E38" s="57">
-        <v>996993.00</v>
+        <v>4713892.00</v>
       </c>
       <c t="n" r="F38">
-        <v>64.4</v>
+        <v>85.3</v>
       </c>
       <c r="H38" s="66">
-        <v>2.05</v>
+        <v>2.27</v>
       </c>
       <c t="inlineStr" r="I38">
         <is>
@@ -2314,16 +2314,16 @@
         <v>100</v>
       </c>
       <c r="O38" s="66">
-        <v>-16.95</v>
+        <v>26.48</v>
       </c>
       <c r="P38" s="65">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="R38" s="66">
-        <v>0.00</v>
+        <v>14.29</v>
       </c>
       <c r="S38" s="65">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="U38" s="65">
         <v>3</v>
@@ -2340,20 +2340,20 @@
       </c>
       <c t="inlineStr" r="C39">
         <is>
-          <t xml:space="preserve">112 - SORIANA SAN JOSE</t>
+          <t xml:space="preserve">113 - LA PAZ SORIANA</t>
         </is>
       </c>
       <c r="D39" s="57">
-        <v>4022300.51</v>
+        <v>1118017.94</v>
       </c>
       <c r="E39" s="57">
-        <v>4713892.00</v>
+        <v>1844843.00</v>
       </c>
       <c t="n" r="F39">
-        <v>85.3</v>
+        <v>60.6</v>
       </c>
       <c r="H39" s="66">
-        <v>2.27</v>
+        <v>1.84</v>
       </c>
       <c t="inlineStr" r="I39">
         <is>
@@ -2370,19 +2370,19 @@
         <v>100</v>
       </c>
       <c r="O39" s="66">
-        <v>26.48</v>
+        <v>12.56</v>
       </c>
       <c r="P39" s="65">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="R39" s="66">
-        <v>13.33</v>
+        <v>18.18</v>
       </c>
       <c r="S39" s="65">
         <v>0</v>
       </c>
       <c r="U39" s="65">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="40">
@@ -2396,20 +2396,20 @@
       </c>
       <c t="inlineStr" r="C40">
         <is>
-          <t xml:space="preserve">113 - LA PAZ SORIANA</t>
+          <t xml:space="preserve">116 - OBREGON BELLAVISTA</t>
         </is>
       </c>
       <c r="D40" s="57">
-        <v>1118017.94</v>
+        <v>914189.66</v>
       </c>
       <c r="E40" s="57">
-        <v>1844843.00</v>
+        <v>1110021.00</v>
       </c>
       <c t="n" r="F40">
-        <v>60.6</v>
+        <v>82.4</v>
       </c>
       <c r="H40" s="66">
-        <v>1.84</v>
+        <v>2.11</v>
       </c>
       <c t="inlineStr" r="I40">
         <is>
@@ -2420,25 +2420,25 @@
         <v>0</v>
       </c>
       <c r="L40" s="57">
-        <v>0.00</v>
+        <v>-8082.35</v>
       </c>
       <c r="M40" s="65">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="O40" s="66">
-        <v>12.56</v>
+        <v>17.87</v>
       </c>
       <c r="P40" s="65">
         <v>0</v>
       </c>
       <c r="R40" s="66">
-        <v>18.18</v>
+        <v>0.00</v>
       </c>
       <c r="S40" s="65">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="U40" s="65">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="41">
@@ -2452,20 +2452,20 @@
       </c>
       <c t="inlineStr" r="C41">
         <is>
-          <t xml:space="preserve">116 - OBREGON BELLAVISTA</t>
+          <t xml:space="preserve">118 - El Dorado Nvo</t>
         </is>
       </c>
       <c r="D41" s="57">
-        <v>914189.66</v>
+        <v>1361130.23</v>
       </c>
       <c r="E41" s="57">
-        <v>1110021.00</v>
+        <v>1599778.00</v>
       </c>
       <c t="n" r="F41">
-        <v>82.4</v>
+        <v>85.1</v>
       </c>
       <c r="H41" s="66">
-        <v>2.11</v>
+        <v>1.87</v>
       </c>
       <c t="inlineStr" r="I41">
         <is>
@@ -2476,16 +2476,16 @@
         <v>0</v>
       </c>
       <c r="L41" s="57">
-        <v>-8082.35</v>
+        <v>-22.34</v>
       </c>
       <c r="M41" s="65">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="O41" s="66">
-        <v>17.87</v>
+        <v>22.89</v>
       </c>
       <c r="P41" s="65">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="R41" s="66">
         <v>0.00</v>
@@ -2494,7 +2494,7 @@
         <v>100</v>
       </c>
       <c r="U41" s="65">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="42">
@@ -2508,20 +2508,20 @@
       </c>
       <c t="inlineStr" r="C42">
         <is>
-          <t xml:space="preserve">117 - TEPIC FORUM</t>
+          <t xml:space="preserve">119 - TIENDA DIGITAL</t>
         </is>
       </c>
       <c r="D42" s="57">
-        <v>0.00</v>
+        <v>5239224.23</v>
       </c>
       <c r="E42" s="57">
-        <v>1438511.48</v>
-      </c>
-      <c t="n" r="F42">
-        <v>0.0</v>
-      </c>
-      <c r="H42" s="65">
-        <v>0</v>
+        <v>0.00</v>
+      </c>
+      <c r="F42" s="65">
+        <v>0</v>
+      </c>
+      <c r="H42" s="66">
+        <v>2.33</v>
       </c>
       <c t="inlineStr" r="I42">
         <is>
@@ -2538,19 +2538,19 @@
         <v>100</v>
       </c>
       <c r="O42" s="66">
-        <v>0.00</v>
+        <v>-65.92</v>
       </c>
       <c r="P42" s="65">
         <v>0</v>
       </c>
-      <c r="R42" s="65">
-        <v>0</v>
+      <c r="R42" s="66">
+        <v>0.00</v>
       </c>
       <c r="S42" s="65">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="U42" s="65">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="43">
@@ -2564,20 +2564,20 @@
       </c>
       <c t="inlineStr" r="C43">
         <is>
-          <t xml:space="preserve">118 - El Dorado Nvo</t>
+          <t xml:space="preserve">126 - Soriana Los Mochis</t>
         </is>
       </c>
       <c r="D43" s="57">
-        <v>1361130.23</v>
+        <v>1290408.57</v>
       </c>
       <c r="E43" s="57">
-        <v>1599778.00</v>
+        <v>1309239.00</v>
       </c>
       <c t="n" r="F43">
-        <v>85.1</v>
+        <v>98.6</v>
       </c>
       <c r="H43" s="66">
-        <v>1.87</v>
+        <v>1.86</v>
       </c>
       <c t="inlineStr" r="I43">
         <is>
@@ -2588,16 +2588,16 @@
         <v>0</v>
       </c>
       <c r="L43" s="57">
-        <v>-22.34</v>
+        <v>-1939.76</v>
       </c>
       <c r="M43" s="65">
         <v>100</v>
       </c>
       <c r="O43" s="66">
-        <v>22.89</v>
+        <v>19.40</v>
       </c>
       <c r="P43" s="65">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="R43" s="66">
         <v>0.00</v>
@@ -2606,7 +2606,7 @@
         <v>100</v>
       </c>
       <c r="U43" s="65">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="44">
@@ -2620,20 +2620,20 @@
       </c>
       <c t="inlineStr" r="C44">
         <is>
-          <t xml:space="preserve">119 - TIENDA DIGITAL</t>
+          <t xml:space="preserve">129 - TIJUANA BENTON</t>
         </is>
       </c>
       <c r="D44" s="57">
-        <v>5239224.23</v>
+        <v>815143.00</v>
       </c>
       <c r="E44" s="57">
-        <v>0.00</v>
-      </c>
-      <c r="F44" s="65">
-        <v>0</v>
+        <v>944015.00</v>
+      </c>
+      <c t="n" r="F44">
+        <v>86.3</v>
       </c>
       <c r="H44" s="66">
-        <v>2.33</v>
+        <v>1.48</v>
       </c>
       <c t="inlineStr" r="I44">
         <is>
@@ -2644,13 +2644,13 @@
         <v>0</v>
       </c>
       <c r="L44" s="57">
-        <v>0.00</v>
+        <v>-4388.83</v>
       </c>
       <c r="M44" s="65">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="O44" s="66">
-        <v>-65.92</v>
+        <v>2.42</v>
       </c>
       <c r="P44" s="65">
         <v>0</v>
@@ -2662,7 +2662,7 @@
         <v>100</v>
       </c>
       <c r="U44" s="65">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="45">
@@ -2676,49 +2676,49 @@
       </c>
       <c t="inlineStr" r="C45">
         <is>
-          <t xml:space="preserve">126 - Soriana Los Mochis</t>
+          <t xml:space="preserve">142 - NAVOLATO CATEDRAL</t>
         </is>
       </c>
       <c r="D45" s="57">
-        <v>1290408.57</v>
+        <v>2426615.05</v>
       </c>
       <c r="E45" s="57">
-        <v>1309239.00</v>
+        <v>2775437.00</v>
       </c>
       <c t="n" r="F45">
-        <v>98.6</v>
+        <v>87.4</v>
       </c>
       <c r="H45" s="66">
-        <v>1.86</v>
+        <v>2.75</v>
       </c>
       <c t="inlineStr" r="I45">
         <is>
-          <t xml:space="preserve">Meta 2.5 · No cumplió</t>
+          <t xml:space="preserve">Meta 2.5 · Cumplió</t>
         </is>
       </c>
       <c r="J45" s="65">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="L45" s="57">
-        <v>-1939.76</v>
+        <v>-5719.50</v>
       </c>
       <c r="M45" s="65">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="O45" s="66">
-        <v>19.40</v>
+        <v>25.01</v>
       </c>
       <c r="P45" s="65">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="R45" s="66">
-        <v>0.00</v>
+        <v>8.33</v>
       </c>
       <c r="S45" s="65">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="U45" s="65">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="46">
@@ -2732,20 +2732,20 @@
       </c>
       <c t="inlineStr" r="C46">
         <is>
-          <t xml:space="preserve">129 - TIJUANA BENTON</t>
+          <t xml:space="preserve">155 - TEPIC HIDALGO</t>
         </is>
       </c>
       <c r="D46" s="57">
-        <v>815143.00</v>
+        <v>1673442.21</v>
       </c>
       <c r="E46" s="57">
-        <v>944015.00</v>
+        <v>2090321.00</v>
       </c>
       <c t="n" r="F46">
-        <v>86.3</v>
+        <v>80.1</v>
       </c>
       <c r="H46" s="66">
-        <v>1.48</v>
+        <v>2.02</v>
       </c>
       <c t="inlineStr" r="I46">
         <is>
@@ -2756,25 +2756,25 @@
         <v>0</v>
       </c>
       <c r="L46" s="57">
-        <v>-4388.83</v>
+        <v>0.00</v>
       </c>
       <c r="M46" s="65">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="O46" s="66">
-        <v>2.42</v>
+        <v>24.07</v>
       </c>
       <c r="P46" s="65">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="R46" s="66">
-        <v>0.00</v>
+        <v>30.00</v>
       </c>
       <c r="S46" s="65">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="U46" s="65">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="47">
@@ -2788,49 +2788,49 @@
       </c>
       <c t="inlineStr" r="C47">
         <is>
-          <t xml:space="preserve">142 - NAVOLATO CATEDRAL</t>
+          <t xml:space="preserve">172 - TIJUANA CONSTITUCION</t>
         </is>
       </c>
       <c r="D47" s="57">
-        <v>2426615.05</v>
+        <v>909273.20</v>
       </c>
       <c r="E47" s="57">
-        <v>2775437.00</v>
+        <v>1151373.00</v>
       </c>
       <c t="n" r="F47">
-        <v>87.4</v>
+        <v>79.0</v>
       </c>
       <c r="H47" s="66">
-        <v>2.75</v>
+        <v>1.39</v>
       </c>
       <c t="inlineStr" r="I47">
         <is>
-          <t xml:space="preserve">Meta 2.5 · Cumplió</t>
+          <t xml:space="preserve">Meta 2.5 · No cumplió</t>
         </is>
       </c>
       <c r="J47" s="65">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="L47" s="57">
-        <v>-5719.50</v>
+        <v>0.00</v>
       </c>
       <c r="M47" s="65">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="O47" s="66">
-        <v>25.01</v>
+        <v>7.92</v>
       </c>
       <c r="P47" s="65">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="R47" s="66">
-        <v>9.09</v>
+        <v>0.00</v>
       </c>
       <c r="S47" s="65">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="U47" s="65">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="48">
@@ -2844,20 +2844,20 @@
       </c>
       <c t="inlineStr" r="C48">
         <is>
-          <t xml:space="preserve">155 - TEPIC HIDALGO</t>
+          <t xml:space="preserve">177 - MAZATLAN SORIANA STA ROSA</t>
         </is>
       </c>
       <c r="D48" s="57">
-        <v>1673442.21</v>
+        <v>658471.77</v>
       </c>
       <c r="E48" s="57">
-        <v>2090321.00</v>
+        <v>791825.00</v>
       </c>
       <c t="n" r="F48">
-        <v>80.1</v>
+        <v>83.2</v>
       </c>
       <c r="H48" s="66">
-        <v>2.02</v>
+        <v>2.14</v>
       </c>
       <c t="inlineStr" r="I48">
         <is>
@@ -2868,25 +2868,25 @@
         <v>0</v>
       </c>
       <c r="L48" s="57">
-        <v>0.00</v>
+        <v>-281.04</v>
       </c>
       <c r="M48" s="65">
         <v>100</v>
       </c>
       <c r="O48" s="66">
-        <v>24.07</v>
+        <v>-6.17</v>
       </c>
       <c r="P48" s="65">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="R48" s="66">
-        <v>30.00</v>
+        <v>14.29</v>
       </c>
       <c r="S48" s="65">
         <v>0</v>
       </c>
       <c r="U48" s="65">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="49">
@@ -2900,20 +2900,20 @@
       </c>
       <c t="inlineStr" r="C49">
         <is>
-          <t xml:space="preserve">169 - ARJONA CLN</t>
+          <t xml:space="preserve">179 - TIJUANA 2000</t>
         </is>
       </c>
       <c r="D49" s="57">
-        <v>652564.49</v>
+        <v>1777966.41</v>
       </c>
       <c r="E49" s="57">
-        <v>759900.00</v>
+        <v>1863024.00</v>
       </c>
       <c t="n" r="F49">
-        <v>85.9</v>
+        <v>95.4</v>
       </c>
       <c r="H49" s="66">
-        <v>1.86</v>
+        <v>1.76</v>
       </c>
       <c t="inlineStr" r="I49">
         <is>
@@ -2924,13 +2924,13 @@
         <v>0</v>
       </c>
       <c r="L49" s="57">
-        <v>-8198.00</v>
+        <v>0.00</v>
       </c>
       <c r="M49" s="65">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="O49" s="66">
-        <v>-13.61</v>
+        <v>16.70</v>
       </c>
       <c r="P49" s="65">
         <v>0</v>
@@ -2942,7 +2942,7 @@
         <v>100</v>
       </c>
       <c r="U49" s="65">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="50">
@@ -2956,20 +2956,20 @@
       </c>
       <c t="inlineStr" r="C50">
         <is>
-          <t xml:space="preserve">172 - TIJUANA CONSTITUCION</t>
+          <t xml:space="preserve">185 - SAN ISIDRO CLN</t>
         </is>
       </c>
       <c r="D50" s="57">
-        <v>909273.20</v>
+        <v>2127577.80</v>
       </c>
       <c r="E50" s="57">
-        <v>1151373.00</v>
+        <v>2769041.00</v>
       </c>
       <c t="n" r="F50">
-        <v>79.0</v>
+        <v>76.8</v>
       </c>
       <c r="H50" s="66">
-        <v>1.39</v>
+        <v>1.92</v>
       </c>
       <c t="inlineStr" r="I50">
         <is>
@@ -2980,13 +2980,13 @@
         <v>0</v>
       </c>
       <c r="L50" s="57">
-        <v>0.00</v>
+        <v>-6732.19</v>
       </c>
       <c r="M50" s="65">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="O50" s="66">
-        <v>7.92</v>
+        <v>15.06</v>
       </c>
       <c r="P50" s="65">
         <v>0</v>
@@ -2998,7 +2998,7 @@
         <v>100</v>
       </c>
       <c r="U50" s="65">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="51">
@@ -3012,49 +3012,49 @@
       </c>
       <c t="inlineStr" r="C51">
         <is>
-          <t xml:space="preserve">177 - MAZATLAN SORIANA STA ROSA</t>
+          <t xml:space="preserve">192 - MAZATLAN SERDAN</t>
         </is>
       </c>
       <c r="D51" s="57">
-        <v>658471.77</v>
+        <v>1256194.15</v>
       </c>
       <c r="E51" s="57">
-        <v>791825.00</v>
+        <v>1076550.00</v>
       </c>
       <c t="n" r="F51">
-        <v>83.2</v>
+        <v>116.7</v>
       </c>
       <c r="H51" s="66">
-        <v>2.14</v>
+        <v>2.74</v>
       </c>
       <c t="inlineStr" r="I51">
         <is>
-          <t xml:space="preserve">Meta 2.5 · No cumplió</t>
+          <t xml:space="preserve">Meta 2.5 · Cumplió</t>
         </is>
       </c>
       <c r="J51" s="65">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="L51" s="57">
-        <v>-281.04</v>
+        <v>27.00</v>
       </c>
       <c r="M51" s="65">
         <v>100</v>
       </c>
       <c r="O51" s="66">
-        <v>-6.17</v>
+        <v>6.72</v>
       </c>
       <c r="P51" s="65">
         <v>0</v>
       </c>
       <c r="R51" s="66">
-        <v>14.29</v>
+        <v>0.00</v>
       </c>
       <c r="S51" s="65">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="U51" s="65">
-        <v>2</v>
+        <v>9</v>
       </c>
     </row>
     <row r="52">
@@ -3068,20 +3068,20 @@
       </c>
       <c t="inlineStr" r="C52">
         <is>
-          <t xml:space="preserve">179 - TIJUANA 2000</t>
+          <t xml:space="preserve">206 - MAZATLAN SORIANA INSURGENTES</t>
         </is>
       </c>
       <c r="D52" s="57">
-        <v>1777966.41</v>
+        <v>0.00</v>
       </c>
       <c r="E52" s="57">
-        <v>1863024.00</v>
+        <v>587313.18</v>
       </c>
       <c t="n" r="F52">
-        <v>95.4</v>
-      </c>
-      <c r="H52" s="66">
-        <v>1.76</v>
+        <v>0.0</v>
+      </c>
+      <c r="H52" s="65">
+        <v>0</v>
       </c>
       <c t="inlineStr" r="I52">
         <is>
@@ -3098,19 +3098,19 @@
         <v>100</v>
       </c>
       <c r="O52" s="66">
-        <v>16.70</v>
+        <v>0.00</v>
       </c>
       <c r="P52" s="65">
         <v>0</v>
       </c>
-      <c r="R52" s="66">
-        <v>0.00</v>
+      <c r="R52" s="65">
+        <v>0</v>
       </c>
       <c r="S52" s="65">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="U52" s="65">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="53">
@@ -3124,20 +3124,20 @@
       </c>
       <c t="inlineStr" r="C53">
         <is>
-          <t xml:space="preserve">185 - SAN ISIDRO CLN</t>
+          <t xml:space="preserve">209 - TIJUANA SENDERO</t>
         </is>
       </c>
       <c r="D53" s="57">
-        <v>2127577.80</v>
+        <v>928802.49</v>
       </c>
       <c r="E53" s="57">
-        <v>2769041.00</v>
+        <v>990889.00</v>
       </c>
       <c t="n" r="F53">
-        <v>76.8</v>
+        <v>93.7</v>
       </c>
       <c r="H53" s="66">
-        <v>1.92</v>
+        <v>1.68</v>
       </c>
       <c t="inlineStr" r="I53">
         <is>
@@ -3148,13 +3148,13 @@
         <v>0</v>
       </c>
       <c r="L53" s="57">
-        <v>-6732.19</v>
+        <v>0.00</v>
       </c>
       <c r="M53" s="65">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="O53" s="66">
-        <v>15.06</v>
+        <v>6.78</v>
       </c>
       <c r="P53" s="65">
         <v>0</v>
@@ -3166,7 +3166,7 @@
         <v>100</v>
       </c>
       <c r="U53" s="65">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="54">
@@ -3180,49 +3180,49 @@
       </c>
       <c t="inlineStr" r="C54">
         <is>
-          <t xml:space="preserve">192 - MAZATLAN SERDAN</t>
+          <t xml:space="preserve">212 - ENSENADA RUIZ</t>
         </is>
       </c>
       <c r="D54" s="57">
-        <v>1256194.15</v>
+        <v>1150510.24</v>
       </c>
       <c r="E54" s="57">
-        <v>1076550.00</v>
+        <v>1912221.00</v>
       </c>
       <c t="n" r="F54">
-        <v>116.7</v>
+        <v>60.2</v>
       </c>
       <c r="H54" s="66">
-        <v>2.74</v>
+        <v>2.24</v>
       </c>
       <c t="inlineStr" r="I54">
         <is>
-          <t xml:space="preserve">Meta 2.5 · Cumplió</t>
+          <t xml:space="preserve">Meta 2.5 · No cumplió</t>
         </is>
       </c>
       <c r="J54" s="65">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="L54" s="57">
-        <v>27.00</v>
+        <v>-1104.99</v>
       </c>
       <c r="M54" s="65">
         <v>100</v>
       </c>
       <c r="O54" s="66">
-        <v>6.72</v>
+        <v>13.23</v>
       </c>
       <c r="P54" s="65">
         <v>0</v>
       </c>
       <c r="R54" s="66">
-        <v>0.00</v>
+        <v>12.50</v>
       </c>
       <c r="S54" s="65">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="U54" s="65">
-        <v>9</v>
+        <v>2</v>
       </c>
     </row>
     <row r="55">
@@ -3236,20 +3236,20 @@
       </c>
       <c t="inlineStr" r="C55">
         <is>
-          <t xml:space="preserve">206 - MAZATLAN SORIANA INSURGENTES</t>
+          <t xml:space="preserve">215 - SORIANA 6 DE ABRIL CABORCA</t>
         </is>
       </c>
       <c r="D55" s="57">
-        <v>0.00</v>
+        <v>1498534.72</v>
       </c>
       <c r="E55" s="57">
-        <v>587313.18</v>
+        <v>2138234.00</v>
       </c>
       <c t="n" r="F55">
-        <v>0.0</v>
-      </c>
-      <c r="H55" s="65">
-        <v>0</v>
+        <v>70.1</v>
+      </c>
+      <c r="H55" s="66">
+        <v>1.66</v>
       </c>
       <c t="inlineStr" r="I55">
         <is>
@@ -3266,19 +3266,19 @@
         <v>100</v>
       </c>
       <c r="O55" s="66">
-        <v>0.00</v>
+        <v>25.49</v>
       </c>
       <c r="P55" s="65">
-        <v>0</v>
-      </c>
-      <c r="R55" s="65">
-        <v>0</v>
+        <v>100</v>
+      </c>
+      <c r="R55" s="66">
+        <v>0.00</v>
       </c>
       <c r="S55" s="65">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="U55" s="65">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="56">
@@ -3292,20 +3292,20 @@
       </c>
       <c t="inlineStr" r="C56">
         <is>
-          <t xml:space="preserve">209 - TIJUANA SENDERO</t>
+          <t xml:space="preserve">217 - ENSENADA COMERCIAL</t>
         </is>
       </c>
       <c r="D56" s="57">
-        <v>928802.49</v>
+        <v>821018.55</v>
       </c>
       <c r="E56" s="57">
-        <v>990889.00</v>
+        <v>1403348.00</v>
       </c>
       <c t="n" r="F56">
-        <v>93.7</v>
-      </c>
-      <c r="H56" s="66">
-        <v>1.68</v>
+        <v>58.5</v>
+      </c>
+      <c t="n" r="H56">
+        <v>1.6</v>
       </c>
       <c t="inlineStr" r="I56">
         <is>
@@ -3316,25 +3316,25 @@
         <v>0</v>
       </c>
       <c r="L56" s="57">
-        <v>0.00</v>
+        <v>-12757.57</v>
       </c>
       <c r="M56" s="65">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="O56" s="66">
-        <v>6.78</v>
+        <v>14.05</v>
       </c>
       <c r="P56" s="65">
         <v>0</v>
       </c>
       <c r="R56" s="66">
-        <v>0.00</v>
+        <v>12.50</v>
       </c>
       <c r="S56" s="65">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="U56" s="65">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="57">
@@ -3348,20 +3348,20 @@
       </c>
       <c t="inlineStr" r="C57">
         <is>
-          <t xml:space="preserve">212 - ENSENADA RUIZ</t>
+          <t xml:space="preserve">242 - PABELLON CULIACAN</t>
         </is>
       </c>
       <c r="D57" s="57">
-        <v>1150510.24</v>
+        <v>833939.14</v>
       </c>
       <c r="E57" s="57">
-        <v>1912221.00</v>
+        <v>1243721.00</v>
       </c>
       <c t="n" r="F57">
-        <v>60.2</v>
+        <v>67.1</v>
       </c>
       <c r="H57" s="66">
-        <v>2.24</v>
+        <v>1.71</v>
       </c>
       <c t="inlineStr" r="I57">
         <is>
@@ -3372,25 +3372,25 @@
         <v>0</v>
       </c>
       <c r="L57" s="57">
-        <v>-1104.99</v>
+        <v>0.00</v>
       </c>
       <c r="M57" s="65">
         <v>100</v>
       </c>
       <c r="O57" s="66">
-        <v>13.23</v>
+        <v>7.03</v>
       </c>
       <c r="P57" s="65">
         <v>0</v>
       </c>
       <c r="R57" s="66">
-        <v>12.50</v>
+        <v>0.00</v>
       </c>
       <c r="S57" s="65">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="U57" s="65">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="58">
@@ -3404,20 +3404,20 @@
       </c>
       <c t="inlineStr" r="C58">
         <is>
-          <t xml:space="preserve">215 - SORIANA 6 DE ABRIL CABORCA</t>
+          <t xml:space="preserve">251 - MEXICALI SENDEROS</t>
         </is>
       </c>
       <c r="D58" s="57">
-        <v>1498534.72</v>
+        <v>1288532.44</v>
       </c>
       <c r="E58" s="57">
-        <v>2138234.00</v>
+        <v>1838412.00</v>
       </c>
       <c t="n" r="F58">
         <v>70.1</v>
       </c>
       <c r="H58" s="66">
-        <v>1.66</v>
+        <v>1.74</v>
       </c>
       <c t="inlineStr" r="I58">
         <is>
@@ -3428,25 +3428,25 @@
         <v>0</v>
       </c>
       <c r="L58" s="57">
-        <v>0.00</v>
+        <v>-9182.98</v>
       </c>
       <c r="M58" s="65">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="O58" s="66">
-        <v>25.49</v>
+        <v>17.35</v>
       </c>
       <c r="P58" s="65">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="R58" s="66">
-        <v>0.00</v>
+        <v>12.50</v>
       </c>
       <c r="S58" s="65">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="U58" s="65">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="59">
@@ -3460,20 +3460,20 @@
       </c>
       <c t="inlineStr" r="C59">
         <is>
-          <t xml:space="preserve">217 - ENSENADA COMERCIAL</t>
+          <t xml:space="preserve">256 - SORIANA CARIBE CABOS</t>
         </is>
       </c>
       <c r="D59" s="57">
-        <v>821018.55</v>
+        <v>2245961.87</v>
       </c>
       <c r="E59" s="57">
-        <v>1403348.00</v>
+        <v>2566802.00</v>
       </c>
       <c t="n" r="F59">
-        <v>58.5</v>
-      </c>
-      <c t="n" r="H59">
-        <v>1.6</v>
+        <v>87.5</v>
+      </c>
+      <c r="H59" s="66">
+        <v>1.83</v>
       </c>
       <c t="inlineStr" r="I59">
         <is>
@@ -3484,25 +3484,25 @@
         <v>0</v>
       </c>
       <c r="L59" s="57">
-        <v>-12757.57</v>
+        <v>0.00</v>
       </c>
       <c r="M59" s="65">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="O59" s="66">
-        <v>14.05</v>
+        <v>24.29</v>
       </c>
       <c r="P59" s="65">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="R59" s="66">
-        <v>25.00</v>
+        <v>0.00</v>
       </c>
       <c r="S59" s="65">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="U59" s="65">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="60">
@@ -3516,20 +3516,20 @@
       </c>
       <c t="inlineStr" r="C60">
         <is>
-          <t xml:space="preserve">225 - LA PRINCIPAL 2 CLN</t>
+          <t xml:space="preserve">258 - GUASAVE PLAZA LEY</t>
         </is>
       </c>
       <c r="D60" s="57">
-        <v>86943.19</v>
+        <v>686832.57</v>
       </c>
       <c r="E60" s="57">
-        <v>83565.00</v>
+        <v>745171.00</v>
       </c>
       <c t="n" r="F60">
-        <v>104.0</v>
+        <v>92.2</v>
       </c>
       <c r="H60" s="66">
-        <v>1.38</v>
+        <v>1.88</v>
       </c>
       <c t="inlineStr" r="I60">
         <is>
@@ -3540,25 +3540,25 @@
         <v>0</v>
       </c>
       <c r="L60" s="57">
-        <v>0.00</v>
+        <v>-681.16</v>
       </c>
       <c r="M60" s="65">
         <v>100</v>
       </c>
       <c r="O60" s="66">
-        <v>-6.37</v>
+        <v>2.85</v>
       </c>
       <c r="P60" s="65">
         <v>0</v>
       </c>
-      <c r="R60" s="65">
-        <v>0</v>
+      <c r="R60" s="66">
+        <v>0.00</v>
       </c>
       <c r="S60" s="65">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="U60" s="65">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="61">
@@ -3572,20 +3572,20 @@
       </c>
       <c t="inlineStr" r="C61">
         <is>
-          <t xml:space="preserve">242 - PABELLON CULIACAN</t>
+          <t xml:space="preserve">263 - VALLARTA CARACOL</t>
         </is>
       </c>
       <c r="D61" s="57">
-        <v>833939.14</v>
+        <v>934983.81</v>
       </c>
       <c r="E61" s="57">
-        <v>1243721.00</v>
+        <v>1304225.00</v>
       </c>
       <c t="n" r="F61">
-        <v>67.1</v>
+        <v>71.7</v>
       </c>
       <c r="H61" s="66">
-        <v>1.71</v>
+        <v>1.79</v>
       </c>
       <c t="inlineStr" r="I61">
         <is>
@@ -3596,25 +3596,25 @@
         <v>0</v>
       </c>
       <c r="L61" s="57">
-        <v>0.00</v>
+        <v>-38.72</v>
       </c>
       <c r="M61" s="65">
         <v>100</v>
       </c>
       <c r="O61" s="66">
-        <v>7.03</v>
+        <v>9.82</v>
       </c>
       <c r="P61" s="65">
         <v>0</v>
       </c>
       <c r="R61" s="66">
-        <v>0.00</v>
+        <v>14.29</v>
       </c>
       <c r="S61" s="65">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="U61" s="65">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="62">
@@ -3628,20 +3628,20 @@
       </c>
       <c t="inlineStr" r="C62">
         <is>
-          <t xml:space="preserve">251 - MEXICALI SENDEROS</t>
+          <t xml:space="preserve">270 - MEXICALI CACHANILLA</t>
         </is>
       </c>
       <c r="D62" s="57">
-        <v>1288532.44</v>
+        <v>1275749.93</v>
       </c>
       <c r="E62" s="57">
-        <v>1838412.00</v>
+        <v>1818043.00</v>
       </c>
       <c t="n" r="F62">
-        <v>70.1</v>
-      </c>
-      <c r="H62" s="66">
-        <v>1.74</v>
+        <v>70.2</v>
+      </c>
+      <c t="n" r="H62">
+        <v>1.6</v>
       </c>
       <c t="inlineStr" r="I62">
         <is>
@@ -3652,13 +3652,13 @@
         <v>0</v>
       </c>
       <c r="L62" s="57">
-        <v>-9182.98</v>
+        <v>124.11</v>
       </c>
       <c r="M62" s="65">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="O62" s="66">
-        <v>17.35</v>
+        <v>14.80</v>
       </c>
       <c r="P62" s="65">
         <v>0</v>
@@ -3670,7 +3670,7 @@
         <v>0</v>
       </c>
       <c r="U62" s="65">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="63">
@@ -3684,20 +3684,20 @@
       </c>
       <c t="inlineStr" r="C63">
         <is>
-          <t xml:space="preserve">256 - SORIANA CARIBE CABOS</t>
+          <t xml:space="preserve">301 - TIJUANA CATEDRAL</t>
         </is>
       </c>
       <c r="D63" s="57">
-        <v>2245961.87</v>
+        <v>728746.42</v>
       </c>
       <c r="E63" s="57">
-        <v>2566802.00</v>
+        <v>806485.00</v>
       </c>
       <c t="n" r="F63">
-        <v>87.5</v>
+        <v>90.4</v>
       </c>
       <c r="H63" s="66">
-        <v>1.83</v>
+        <v>1.52</v>
       </c>
       <c t="inlineStr" r="I63">
         <is>
@@ -3714,19 +3714,19 @@
         <v>100</v>
       </c>
       <c r="O63" s="66">
-        <v>24.29</v>
+        <v>7.87</v>
       </c>
       <c r="P63" s="65">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="R63" s="66">
-        <v>8.33</v>
+        <v>11.11</v>
       </c>
       <c r="S63" s="65">
         <v>0</v>
       </c>
       <c r="U63" s="65">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="64">
@@ -3740,20 +3740,20 @@
       </c>
       <c t="inlineStr" r="C64">
         <is>
-          <t xml:space="preserve">258 - GUASAVE PLAZA LEY</t>
+          <t xml:space="preserve">303 - PABELLON ROSARITO</t>
         </is>
       </c>
       <c r="D64" s="57">
-        <v>686832.57</v>
+        <v>1020271.11</v>
       </c>
       <c r="E64" s="57">
-        <v>745171.00</v>
+        <v>1264873.00</v>
       </c>
       <c t="n" r="F64">
-        <v>92.2</v>
-      </c>
-      <c r="H64" s="66">
-        <v>1.88</v>
+        <v>80.7</v>
+      </c>
+      <c t="n" r="H64">
+        <v>1.7</v>
       </c>
       <c t="inlineStr" r="I64">
         <is>
@@ -3764,13 +3764,13 @@
         <v>0</v>
       </c>
       <c r="L64" s="57">
-        <v>-681.16</v>
+        <v>-1030.91</v>
       </c>
       <c r="M64" s="65">
         <v>100</v>
       </c>
       <c r="O64" s="66">
-        <v>2.85</v>
+        <v>-1.56</v>
       </c>
       <c r="P64" s="65">
         <v>0</v>
@@ -3796,20 +3796,20 @@
       </c>
       <c t="inlineStr" r="C65">
         <is>
-          <t xml:space="preserve">263 - VALLARTA CARACOL</t>
+          <t xml:space="preserve">310 - CENTRO 19 GUAYMAS</t>
         </is>
       </c>
       <c r="D65" s="57">
-        <v>934983.81</v>
+        <v>331710.11</v>
       </c>
       <c r="E65" s="57">
-        <v>1304225.00</v>
+        <v>642150.00</v>
       </c>
       <c t="n" r="F65">
-        <v>71.7</v>
+        <v>51.7</v>
       </c>
       <c r="H65" s="66">
-        <v>1.79</v>
+        <v>1.67</v>
       </c>
       <c t="inlineStr" r="I65">
         <is>
@@ -3820,19 +3820,19 @@
         <v>0</v>
       </c>
       <c r="L65" s="57">
-        <v>-38.72</v>
+        <v>0.00</v>
       </c>
       <c r="M65" s="65">
         <v>100</v>
       </c>
       <c r="O65" s="66">
-        <v>9.82</v>
+        <v>-12.85</v>
       </c>
       <c r="P65" s="65">
         <v>0</v>
       </c>
       <c r="R65" s="66">
-        <v>14.29</v>
+        <v>16.67</v>
       </c>
       <c r="S65" s="65">
         <v>0</v>
@@ -3852,20 +3852,20 @@
       </c>
       <c t="inlineStr" r="C66">
         <is>
-          <t xml:space="preserve">270 - MEXICALI CACHANILLA</t>
+          <t xml:space="preserve">319 - VISTA HERMOSA SAN JOSE</t>
         </is>
       </c>
       <c r="D66" s="57">
-        <v>1275749.93</v>
+        <v>1815555.52</v>
       </c>
       <c r="E66" s="57">
-        <v>1818043.00</v>
+        <v>2186881.00</v>
       </c>
       <c t="n" r="F66">
-        <v>70.2</v>
-      </c>
-      <c t="n" r="H66">
-        <v>1.6</v>
+        <v>83.0</v>
+      </c>
+      <c r="H66" s="66">
+        <v>2.14</v>
       </c>
       <c t="inlineStr" r="I66">
         <is>
@@ -3876,19 +3876,19 @@
         <v>0</v>
       </c>
       <c r="L66" s="57">
-        <v>124.11</v>
+        <v>0.00</v>
       </c>
       <c r="M66" s="65">
         <v>100</v>
       </c>
       <c r="O66" s="66">
-        <v>14.80</v>
+        <v>17.37</v>
       </c>
       <c r="P66" s="65">
         <v>0</v>
       </c>
       <c r="R66" s="66">
-        <v>12.50</v>
+        <v>20.00</v>
       </c>
       <c r="S66" s="65">
         <v>0</v>
@@ -3908,20 +3908,20 @@
       </c>
       <c t="inlineStr" r="C67">
         <is>
-          <t xml:space="preserve">301 - TIJUANA CATEDRAL</t>
+          <t xml:space="preserve">326 - PLAZA DEL SOL GUADALAJARA</t>
         </is>
       </c>
       <c r="D67" s="57">
-        <v>728746.42</v>
+        <v>559237.03</v>
       </c>
       <c r="E67" s="57">
-        <v>806485.00</v>
+        <v>418066.00</v>
       </c>
       <c t="n" r="F67">
-        <v>90.4</v>
+        <v>133.8</v>
       </c>
       <c r="H67" s="66">
-        <v>1.52</v>
+        <v>2.15</v>
       </c>
       <c t="inlineStr" r="I67">
         <is>
@@ -3938,299 +3938,19 @@
         <v>100</v>
       </c>
       <c r="O67" s="66">
-        <v>7.87</v>
+        <v>-53.10</v>
       </c>
       <c r="P67" s="65">
         <v>0</v>
       </c>
       <c r="R67" s="66">
-        <v>11.11</v>
+        <v>25.00</v>
       </c>
       <c r="S67" s="65">
         <v>0</v>
       </c>
       <c r="U67" s="65">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" s="65">
-        <v>66</v>
-      </c>
-      <c t="inlineStr" r="B68">
-        <is>
-          <t xml:space="preserve">Calzapato</t>
-        </is>
-      </c>
-      <c t="inlineStr" r="C68">
-        <is>
-          <t xml:space="preserve">303 - PABELLON ROSARITO</t>
-        </is>
-      </c>
-      <c r="D68" s="57">
-        <v>1020271.11</v>
-      </c>
-      <c r="E68" s="57">
-        <v>1264873.00</v>
-      </c>
-      <c t="n" r="F68">
-        <v>80.7</v>
-      </c>
-      <c t="n" r="H68">
-        <v>1.7</v>
-      </c>
-      <c t="inlineStr" r="I68">
-        <is>
-          <t xml:space="preserve">Meta 2.5 · No cumplió</t>
-        </is>
-      </c>
-      <c r="J68" s="65">
-        <v>0</v>
-      </c>
-      <c r="L68" s="57">
-        <v>-1030.91</v>
-      </c>
-      <c r="M68" s="65">
-        <v>100</v>
-      </c>
-      <c r="O68" s="66">
-        <v>-1.56</v>
-      </c>
-      <c r="P68" s="65">
-        <v>0</v>
-      </c>
-      <c r="R68" s="66">
-        <v>0.00</v>
-      </c>
-      <c r="S68" s="65">
-        <v>100</v>
-      </c>
-      <c r="U68" s="65">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" s="65">
-        <v>67</v>
-      </c>
-      <c t="inlineStr" r="B69">
-        <is>
-          <t xml:space="preserve">Calzapato</t>
-        </is>
-      </c>
-      <c t="inlineStr" r="C69">
-        <is>
-          <t xml:space="preserve">310 - CENTRO 19 GUAYMAS</t>
-        </is>
-      </c>
-      <c r="D69" s="57">
-        <v>331710.11</v>
-      </c>
-      <c r="E69" s="57">
-        <v>642150.00</v>
-      </c>
-      <c t="n" r="F69">
-        <v>51.7</v>
-      </c>
-      <c r="H69" s="66">
-        <v>1.67</v>
-      </c>
-      <c t="inlineStr" r="I69">
-        <is>
-          <t xml:space="preserve">Meta 2.5 · No cumplió</t>
-        </is>
-      </c>
-      <c r="J69" s="65">
-        <v>0</v>
-      </c>
-      <c r="L69" s="57">
-        <v>0.00</v>
-      </c>
-      <c r="M69" s="65">
-        <v>100</v>
-      </c>
-      <c r="O69" s="66">
-        <v>-12.85</v>
-      </c>
-      <c r="P69" s="65">
-        <v>0</v>
-      </c>
-      <c r="R69" s="66">
-        <v>16.67</v>
-      </c>
-      <c r="S69" s="65">
-        <v>0</v>
-      </c>
-      <c r="U69" s="65">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" s="65">
-        <v>68</v>
-      </c>
-      <c t="inlineStr" r="B70">
-        <is>
-          <t xml:space="preserve">Calzapato</t>
-        </is>
-      </c>
-      <c t="inlineStr" r="C70">
-        <is>
-          <t xml:space="preserve">319 - VISTA HERMOSA SAN JOSE</t>
-        </is>
-      </c>
-      <c r="D70" s="57">
-        <v>1815555.52</v>
-      </c>
-      <c r="E70" s="57">
-        <v>2186881.00</v>
-      </c>
-      <c t="n" r="F70">
-        <v>83.0</v>
-      </c>
-      <c r="H70" s="66">
-        <v>2.14</v>
-      </c>
-      <c t="inlineStr" r="I70">
-        <is>
-          <t xml:space="preserve">Meta 2.5 · No cumplió</t>
-        </is>
-      </c>
-      <c r="J70" s="65">
-        <v>0</v>
-      </c>
-      <c r="L70" s="57">
-        <v>0.00</v>
-      </c>
-      <c r="M70" s="65">
-        <v>100</v>
-      </c>
-      <c r="O70" s="66">
-        <v>17.37</v>
-      </c>
-      <c r="P70" s="65">
-        <v>0</v>
-      </c>
-      <c r="R70" s="66">
-        <v>20.00</v>
-      </c>
-      <c r="S70" s="65">
-        <v>0</v>
-      </c>
-      <c r="U70" s="65">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" s="65">
-        <v>69</v>
-      </c>
-      <c t="inlineStr" r="B71">
-        <is>
-          <t xml:space="preserve">Calzapato</t>
-        </is>
-      </c>
-      <c t="inlineStr" r="C71">
-        <is>
-          <t xml:space="preserve">326 - PLAZA DEL SOL GUADALAJARA</t>
-        </is>
-      </c>
-      <c r="D71" s="57">
-        <v>559237.03</v>
-      </c>
-      <c r="E71" s="57">
-        <v>418066.00</v>
-      </c>
-      <c t="n" r="F71">
-        <v>133.8</v>
-      </c>
-      <c r="H71" s="66">
-        <v>2.15</v>
-      </c>
-      <c t="inlineStr" r="I71">
-        <is>
-          <t xml:space="preserve">Meta 2.5 · No cumplió</t>
-        </is>
-      </c>
-      <c r="J71" s="65">
-        <v>0</v>
-      </c>
-      <c r="L71" s="57">
-        <v>0.00</v>
-      </c>
-      <c r="M71" s="65">
-        <v>100</v>
-      </c>
-      <c r="O71" s="66">
-        <v>-53.10</v>
-      </c>
-      <c r="P71" s="65">
-        <v>0</v>
-      </c>
-      <c r="R71" s="66">
-        <v>20.00</v>
-      </c>
-      <c r="S71" s="65">
-        <v>0</v>
-      </c>
-      <c r="U71" s="65">
         <v>4</v>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" s="65">
-        <v>70</v>
-      </c>
-      <c t="inlineStr" r="B72">
-        <is>
-          <t xml:space="preserve">Calzapato</t>
-        </is>
-      </c>
-      <c t="inlineStr" r="C72">
-        <is>
-          <t xml:space="preserve">357 - SORIANA TERRAZAS MEXICALI</t>
-        </is>
-      </c>
-      <c r="D72" s="57">
-        <v>128209.79</v>
-      </c>
-      <c r="E72" s="57">
-        <v>391423.00</v>
-      </c>
-      <c t="n" r="F72">
-        <v>32.8</v>
-      </c>
-      <c r="H72" s="66">
-        <v>1.43</v>
-      </c>
-      <c t="inlineStr" r="I72">
-        <is>
-          <t xml:space="preserve">Meta 2.5 · No cumplió</t>
-        </is>
-      </c>
-      <c r="J72" s="65">
-        <v>0</v>
-      </c>
-      <c r="L72" s="57">
-        <v>0.00</v>
-      </c>
-      <c r="M72" s="65">
-        <v>100</v>
-      </c>
-      <c r="O72" s="66">
-        <v>-111.46</v>
-      </c>
-      <c r="P72" s="65">
-        <v>0</v>
-      </c>
-      <c r="R72" s="66">
-        <v>40.00</v>
-      </c>
-      <c r="S72" s="65">
-        <v>0</v>
-      </c>
-      <c r="U72" s="65">
-        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>